<commit_message>
Remapped pins to have WS2812 DOUT and PWM CH1 on the same pin
</commit_message>
<xml_diff>
--- a/Hardware/Controller/JLC_PCBA_CPL-DALI_EVG_Controller(V0.1).xlsx
+++ b/Hardware/Controller/JLC_PCBA_CPL-DALI_EVG_Controller(V0.1).xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="0" defaultRowHeight="12.75"/>
   <cols>
     <col width="16.796875" customWidth="1" style="28" min="1" max="1"/>
@@ -681,12 +681,12 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>32.25</t>
         </is>
       </c>
       <c r="C2" s="18" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>10.75</t>
         </is>
       </c>
       <c r="D2" s="18" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="E2" s="18" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F2" s="18" t="inlineStr">
@@ -723,22 +723,22 @@
       </c>
       <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>13.919</t>
+          <t>44.5</t>
         </is>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>14.503</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E3" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F3" s="19" t="inlineStr">
@@ -765,22 +765,22 @@
       </c>
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>16.104</t>
+          <t>20.25</t>
         </is>
       </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
-          <t>11.608</t>
+          <t>9.75</t>
         </is>
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F4" s="19" t="inlineStr">
@@ -802,27 +802,27 @@
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>22.25</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E5" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F5" s="19" t="inlineStr">
@@ -844,27 +844,27 @@
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>C11</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>34.25</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F6" s="19" t="inlineStr">
@@ -874,39 +874,39 @@
       </c>
       <c r="G6" s="19" t="inlineStr">
         <is>
-          <t>10uF/50V</t>
+          <t>100nF</t>
         </is>
       </c>
       <c r="H6" s="19" t="inlineStr">
         <is>
-          <t>C1206</t>
+          <t>C0402</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C12</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>-0.559</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>18.999</t>
+          <t>21.75</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
@@ -916,39 +916,39 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>100nF</t>
+          <t>10uF/50V</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>C0402</t>
+          <t>C1206</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>C14</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>-5.41</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>8.128</t>
+          <t>17.75</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F8" s="19" t="inlineStr">
@@ -970,27 +970,27 @@
     <row r="9">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>-5.4</t>
+          <t>30.1</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
@@ -1012,27 +1012,27 @@
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>12.25</t>
+          <t>29.1</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>19.5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
@@ -1047,34 +1047,34 @@
       </c>
       <c r="H10" s="19" t="inlineStr">
         <is>
-          <t>C0603</t>
+          <t>C0402</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>32.36</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>20.091</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F11" s="19" t="inlineStr">
@@ -1084,29 +1084,29 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>22uF</t>
+          <t>100nF/50V</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>C0805</t>
+          <t>C0402</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C17</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F12" s="19" t="inlineStr">
@@ -1131,24 +1131,24 @@
       </c>
       <c r="H12" s="19" t="inlineStr">
         <is>
-          <t>C0805</t>
+          <t>C0603</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>14.15</t>
+          <t>29.5</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F13" s="19" t="inlineStr">
@@ -1168,39 +1168,39 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>10uF/50V</t>
+          <t>22uF</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>C1206</t>
+          <t>C0603</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>C20</t>
+          <t>C19</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>10.25</t>
+          <t>30.988</t>
         </is>
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>18.339</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F14" s="19" t="inlineStr">
@@ -1210,12 +1210,12 @@
       </c>
       <c r="G14" s="19" t="inlineStr">
         <is>
-          <t>10uF</t>
+          <t>10uF/50V</t>
         </is>
       </c>
       <c r="H14" s="19" t="inlineStr">
         <is>
-          <t>C0805</t>
+          <t>C1206</t>
         </is>
       </c>
     </row>
@@ -1227,22 +1227,22 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>14.859</t>
+          <t>35.5</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>6.756</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F15" s="19" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>10.965</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>17.12</t>
+          <t>20.75</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="H16" s="19" t="inlineStr">
         <is>
-          <t>SMD_Elko_10x10x10.5</t>
+          <t>CAPR-5mm</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>28.7</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="E17" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F17" s="19" t="inlineStr">
@@ -1353,12 +1353,12 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>32.3</t>
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="E18" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F18" s="19" t="inlineStr">
@@ -1395,22 +1395,22 @@
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>19.05</t>
+          <t>41.25</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>14.376</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F19" s="19" t="inlineStr">
@@ -1432,27 +1432,27 @@
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F20" s="19" t="inlineStr">
@@ -1462,34 +1462,34 @@
       </c>
       <c r="G20" s="19" t="inlineStr">
         <is>
-          <t>B5819W SL</t>
+          <t>BAV99</t>
         </is>
       </c>
       <c r="H20" s="19" t="inlineStr">
         <is>
-          <t>SOD-123</t>
+          <t>SOT23</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>6.274</t>
+          <t>29.5</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>10.262</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E21" s="19" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="F21" s="19" t="inlineStr">
         <is>
-          <t>Not Fitted</t>
+          <t>Fitted</t>
         </is>
       </c>
       <c r="G21" s="19" t="inlineStr">
@@ -1516,27 +1516,27 @@
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>14.75</t>
+          <t>26.25</t>
         </is>
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>13.75</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F22" s="19" t="inlineStr">
@@ -1563,22 +1563,22 @@
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t>2.845</t>
+          <t>24.25</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>17.882</t>
+          <t>13.75</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F23" s="19" t="inlineStr">
@@ -1605,22 +1605,22 @@
       </c>
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>27.94</t>
+          <t>45</t>
         </is>
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>12.446</t>
+          <t>10.5</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F24" s="19" t="inlineStr">
@@ -1647,22 +1647,22 @@
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>28.25</t>
+          <t>45</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>18.827</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F25" s="19" t="inlineStr">
@@ -1684,27 +1684,27 @@
     <row r="26">
       <c r="A26" s="25" t="inlineStr">
         <is>
-          <t>IC1</t>
+          <t>FB1</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F26" s="19" t="inlineStr">
@@ -1714,34 +1714,34 @@
       </c>
       <c r="G26" s="19" t="inlineStr">
         <is>
-          <t>TPS54202</t>
+          <t>GZ1608D601TF</t>
         </is>
       </c>
       <c r="H26" s="19" t="inlineStr">
         <is>
-          <t>SOT23-6</t>
+          <t>0603</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>IC1</t>
         </is>
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>2.08</t>
+          <t>35.5</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>5.223</t>
+          <t>20.75</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
@@ -1751,34 +1751,34 @@
       </c>
       <c r="F27" s="19" t="inlineStr">
         <is>
-          <t>Not Fitted</t>
+          <t>Fitted</t>
         </is>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>USB 3.1 C Receptacle</t>
+          <t>LGS5145</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>SOT95P280X110-6N (SOT23-6L)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="25" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>14.25</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>3.948</t>
         </is>
       </c>
       <c r="D28" s="19" t="inlineStr">
@@ -1793,39 +1793,39 @@
       </c>
       <c r="F28" s="19" t="inlineStr">
         <is>
-          <t>Fitted</t>
+          <t>Not Fitted</t>
         </is>
       </c>
       <c r="G28" s="19" t="inlineStr">
         <is>
-          <t>C720477</t>
+          <t>USB 3.1 C Receptacle</t>
         </is>
       </c>
       <c r="H28" s="19" t="inlineStr">
         <is>
-          <t>TS-1088-AR02016</t>
+          <t>C165948</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="25" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>5.274</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E29" s="19" t="inlineStr">
@@ -1852,27 +1852,27 @@
     <row r="30">
       <c r="A30" s="25" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>-10.367</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>11.625</t>
+          <t>19.25</t>
         </is>
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F30" s="19" t="inlineStr">
@@ -1882,29 +1882,29 @@
       </c>
       <c r="G30" s="19" t="inlineStr">
         <is>
-          <t>C262302</t>
+          <t>C720477</t>
         </is>
       </c>
       <c r="H30" s="19" t="inlineStr">
         <is>
-          <t>CONN-TH-10P_AFC11-S10ICC-00</t>
+          <t>TS-1088-AR02016</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="25" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>-10.375</t>
+          <t>11.625</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>11.125</t>
+          <t>11.625</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="F31" s="19" t="inlineStr">
         <is>
-          <t>Not Fitted</t>
+          <t>Fitted</t>
         </is>
       </c>
       <c r="G31" s="19" t="inlineStr">
@@ -1936,17 +1936,17 @@
     <row r="32">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>9.75</t>
+          <t>12.383</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>15.25</t>
+          <t>11.625</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
@@ -1961,39 +1961,39 @@
       </c>
       <c r="F32" s="19" t="inlineStr">
         <is>
-          <t>Fitted</t>
+          <t>Not Fitted</t>
         </is>
       </c>
       <c r="G32" s="19" t="inlineStr">
         <is>
-          <t>15uH</t>
+          <t>C262302</t>
         </is>
       </c>
       <c r="H32" s="19" t="inlineStr">
         <is>
-          <t>5.8x5.2mm</t>
+          <t>CONN-TH-10P_AFC11-S10ICC-00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="25" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>-0.132</t>
+          <t>32.741</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>15.418</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
@@ -2003,39 +2003,39 @@
       </c>
       <c r="F33" s="19" t="inlineStr">
         <is>
-          <t>Not Fitted</t>
+          <t>Fitted</t>
         </is>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>4 Pin male</t>
+          <t>CMI321609X100KT (10uH)</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>TE_826647-4</t>
+          <t>L1210</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="25" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>29.845</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>14.827</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
@@ -2045,39 +2045,39 @@
       </c>
       <c r="F34" s="19" t="inlineStr">
         <is>
-          <t>Fitted</t>
+          <t>Not Fitted</t>
         </is>
       </c>
       <c r="G34" s="19" t="inlineStr">
         <is>
-          <t>KF2EDGR-3.81-4Pin</t>
+          <t>4 Pin male</t>
         </is>
       </c>
       <c r="H34" s="19" t="inlineStr">
         <is>
-          <t>CONN-TH_4P-P3.81_KF2EDGR-3.81-4P</t>
+          <t>TE_826647-4</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="25" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>-17.5</t>
+          <t>47.75</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>12.287</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
@@ -2104,17 +2104,17 @@
     <row r="36">
       <c r="A36" s="25" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>-14.225</t>
+          <t>5.237</t>
         </is>
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.536</t>
         </is>
       </c>
       <c r="D36" s="19" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F36" s="19" t="inlineStr">
@@ -2134,34 +2134,34 @@
       </c>
       <c r="G36" s="19" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>KF2EDGR-3.5-2Pin</t>
         </is>
       </c>
       <c r="H36" s="19" t="inlineStr">
         <is>
-          <t>TE_826647-4</t>
+          <t>CONN-TH_2P-P3.50_KF2EDGR-3.5</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="25" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
         <is>
-          <t>27.77</t>
+          <t>8.525</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>5.436</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
@@ -2176,39 +2176,39 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>MMBT2222A</t>
+          <t>Header</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>SOT23</t>
+          <t>TE_826647-4</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="25" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
         <is>
-          <t>4.35</t>
+          <t>38.25</t>
         </is>
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>6.325</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F38" s="19" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="G38" s="19" t="inlineStr">
         <is>
-          <t>AO3401A</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="H38" s="19" t="inlineStr">
@@ -2230,27 +2230,27 @@
     <row r="39">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>13.75</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F39" s="19" t="inlineStr">
@@ -2260,39 +2260,39 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>MMBT5401</t>
+          <t>AO3401A</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>SOT23</t>
+          <t>SOT23 Normal</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="25" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>18.25</t>
         </is>
       </c>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F40" s="19" t="inlineStr">
@@ -2302,39 +2302,39 @@
       </c>
       <c r="G40" s="19" t="inlineStr">
         <is>
-          <t>AO3400A</t>
+          <t>MMBT5401</t>
         </is>
       </c>
       <c r="H40" s="19" t="inlineStr">
         <is>
-          <t>SOT23 Normal</t>
+          <t>SOT23 Reverse</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="25" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>20.75</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>17.5</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F41" s="19" t="inlineStr">
@@ -2344,39 +2344,39 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>MMBT5551</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>SOT23 Reverse</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="25" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>27.534</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>2.184</t>
+          <t>10.5</t>
         </is>
       </c>
       <c r="D42" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F42" s="19" t="inlineStr">
@@ -2386,39 +2386,39 @@
       </c>
       <c r="G42" s="19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="H42" s="19" t="inlineStr">
         <is>
-          <t>R1206</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="25" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>24.943</t>
+          <t>39</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>5.029</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F43" s="19" t="inlineStr">
@@ -2428,39 +2428,39 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0805</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>24.943</t>
+          <t>35.75</t>
         </is>
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>4.029</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D44" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E44" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F44" s="19" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="G44" s="19" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="H44" s="19" t="inlineStr">
@@ -2482,27 +2482,27 @@
     <row r="45">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>35.75</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>5.9</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F45" s="19" t="inlineStr">
@@ -2517,24 +2517,24 @@
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>0402</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>4.627</t>
+          <t>14.5</t>
         </is>
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>12.924</t>
+          <t>17.75</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="E46" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F46" s="19" t="inlineStr">
@@ -2554,39 +2554,39 @@
       </c>
       <c r="G46" s="19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="H46" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
         <is>
-          <t>3.527</t>
+          <t>17.75</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>12.924</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F47" s="19" t="inlineStr">
@@ -2596,12 +2596,12 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>22k</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R1206</t>
         </is>
       </c>
     </row>
@@ -2613,22 +2613,22 @@
       </c>
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>-6.446</t>
+          <t>26</t>
         </is>
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9.75</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E48" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F48" s="19" t="inlineStr">
@@ -2655,22 +2655,22 @@
       </c>
       <c r="B49" s="19" t="inlineStr">
         <is>
-          <t>-5.446</t>
+          <t>26</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10.75</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F49" s="19" t="inlineStr">
@@ -2697,22 +2697,22 @@
       </c>
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>14.783</t>
+          <t>41.5</t>
         </is>
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>9.957</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F50" s="19" t="inlineStr">
@@ -2739,22 +2739,22 @@
       </c>
       <c r="B51" s="19" t="inlineStr">
         <is>
-          <t>-0.584</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>18.009</t>
+          <t>19.75</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F51" s="19" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -2781,22 +2781,22 @@
       </c>
       <c r="B52" s="19" t="inlineStr">
         <is>
-          <t>1.301</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>12.399</t>
+          <t>4.25</t>
         </is>
       </c>
       <c r="D52" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F52" s="19" t="inlineStr">
@@ -2823,22 +2823,22 @@
       </c>
       <c r="B53" s="19" t="inlineStr">
         <is>
-          <t>1.301</t>
+          <t>25.5</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>13.399</t>
+          <t>4.25</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F53" s="19" t="inlineStr">
@@ -2865,22 +2865,22 @@
       </c>
       <c r="B54" s="19" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>14.7</t>
+          <t>9.35</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E54" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F54" s="19" t="inlineStr">
@@ -2907,22 +2907,22 @@
       </c>
       <c r="B55" s="19" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>16.2</t>
+          <t>9.35</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F55" s="19" t="inlineStr">
@@ -2949,22 +2949,22 @@
       </c>
       <c r="B56" s="19" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>20.84</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="D56" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E56" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F56" s="19" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="H56" s="19" t="inlineStr">
@@ -2986,27 +2986,27 @@
     <row r="57">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R27</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
         <is>
-          <t>-1.702</t>
+          <t>23.5</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>21.184</t>
+          <t>17.75</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E57" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F57" s="19" t="inlineStr">
@@ -3016,39 +3016,39 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>R27</t>
+          <t>R28</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
         <is>
-          <t>9.119</t>
+          <t>38.5</t>
         </is>
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D58" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E58" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F58" s="19" t="inlineStr">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="H58" s="19" t="inlineStr">
@@ -3070,27 +3070,27 @@
     <row r="59">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>R28</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>7.75</t>
+          <t>12.75</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F59" s="19" t="inlineStr">
@@ -3100,24 +3100,24 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>0402</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R30</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
         <is>
-          <t>12.75</t>
+          <t>37.75</t>
         </is>
       </c>
       <c r="C60" s="19" t="inlineStr">
@@ -3127,12 +3127,12 @@
       </c>
       <c r="D60" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F60" s="19" t="inlineStr">
@@ -3142,39 +3142,39 @@
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="H60" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>R30</t>
+          <t>R31</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
         <is>
-          <t>13.25</t>
+          <t>37.25</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>5.75</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F61" s="19" t="inlineStr">
@@ -3184,39 +3184,39 @@
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>R31</t>
+          <t>R32</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>37.75</t>
         </is>
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>13.25</t>
         </is>
       </c>
       <c r="D62" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F62" s="19" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="G62" s="19" t="inlineStr">
         <is>
-          <t>330k</t>
+          <t>8.2k</t>
         </is>
       </c>
       <c r="H62" s="19" t="inlineStr">
@@ -3238,27 +3238,27 @@
     <row r="63">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>R33</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
         <is>
-          <t>15.008</t>
+          <t>35.75</t>
         </is>
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>3.734</t>
+          <t>5.75</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E63" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F63" s="19" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>220k</t>
+          <t>18k</t>
         </is>
       </c>
       <c r="H63" s="19" t="inlineStr">
@@ -3280,27 +3280,27 @@
     <row r="64">
       <c r="A64" s="25" t="inlineStr">
         <is>
-          <t>R33</t>
+          <t>R41</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
         <is>
-          <t>16.508</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>3.734</t>
+          <t>17.75</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F64" s="19" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="G64" s="19" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H64" s="19" t="inlineStr">
@@ -3322,17 +3322,17 @@
     <row r="65">
       <c r="A65" s="25" t="inlineStr">
         <is>
-          <t>R41</t>
+          <t>R42</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
         <is>
-          <t>4.496</t>
+          <t>26.5</t>
         </is>
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>15.418</t>
+          <t>17.75</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="E65" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F65" s="19" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="G65" s="19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H65" s="19" t="inlineStr">
@@ -3364,22 +3364,22 @@
     <row r="66">
       <c r="A66" s="25" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R46</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
         <is>
-          <t>10.287</t>
+          <t>39.5</t>
         </is>
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>10.008</t>
+          <t>18.75</t>
         </is>
       </c>
       <c r="D66" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E66" s="19" t="inlineStr">
@@ -3389,12 +3389,12 @@
       </c>
       <c r="F66" s="19" t="inlineStr">
         <is>
-          <t>Not Fitted</t>
+          <t>Fitted</t>
         </is>
       </c>
       <c r="G66" s="19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="H66" s="19" t="inlineStr">
@@ -3406,17 +3406,17 @@
     <row r="67">
       <c r="A67" s="25" t="inlineStr">
         <is>
-          <t>R46</t>
+          <t>R47</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>39.5</t>
         </is>
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>19.75</t>
+          <t>21.25</t>
         </is>
       </c>
       <c r="D67" s="19" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="E67" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F67" s="19" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="G67" s="19" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="H67" s="19" t="inlineStr">
@@ -3448,27 +3448,27 @@
     <row r="68">
       <c r="A68" s="25" t="inlineStr">
         <is>
-          <t>R47</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>30.261</t>
         </is>
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>21.75</t>
+          <t>4.671</t>
         </is>
       </c>
       <c r="D68" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>225</t>
         </is>
       </c>
       <c r="E68" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F68" s="19" t="inlineStr">
@@ -3478,34 +3478,34 @@
       </c>
       <c r="G68" s="19" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>CH32V003F4U6</t>
         </is>
       </c>
       <c r="H68" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>QFN-20_L3.0-W3.0-P0.40-TL-EP1.7</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="25" t="inlineStr">
         <is>
-          <t>SB1</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
         <is>
-          <t>-9.315</t>
+          <t>34.75</t>
         </is>
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>17.628</t>
+          <t>9.75</t>
         </is>
       </c>
       <c r="D69" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E69" s="19" t="inlineStr">
@@ -3520,39 +3520,39 @@
       </c>
       <c r="G69" s="19" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>LMV331IDBVRG4</t>
         </is>
       </c>
       <c r="H69" s="19" t="inlineStr">
         <is>
-          <t>SB_0603</t>
+          <t>SOT23-5</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="25" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
         <is>
-          <t>-3.708</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>13.564</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D70" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E70" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F70" s="19" t="inlineStr">
@@ -3562,94 +3562,10 @@
       </c>
       <c r="G70" s="19" t="inlineStr">
         <is>
-          <t>CH32V003F4P6</t>
+          <t>AT24C256C-SSHL-T</t>
         </is>
       </c>
       <c r="H70" s="19" t="inlineStr">
-        <is>
-          <t>SOP65P640X121-20N</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="25" t="inlineStr">
-        <is>
-          <t>U2</t>
-        </is>
-      </c>
-      <c r="B71" s="19" t="inlineStr">
-        <is>
-          <t>9.5</t>
-        </is>
-      </c>
-      <c r="C71" s="19" t="inlineStr">
-        <is>
-          <t>6.25</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
-        <is>
-          <t>270</t>
-        </is>
-      </c>
-      <c r="E71" s="19" t="inlineStr">
-        <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="F71" s="19" t="inlineStr">
-        <is>
-          <t>Fitted</t>
-        </is>
-      </c>
-      <c r="G71" s="19" t="inlineStr">
-        <is>
-          <t>LM393DR2G</t>
-        </is>
-      </c>
-      <c r="H71" s="19" t="inlineStr">
-        <is>
-          <t>SOIC127P600X265-8N (SOIC-8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="25" t="inlineStr">
-        <is>
-          <t>U3</t>
-        </is>
-      </c>
-      <c r="B72" s="19" t="inlineStr">
-        <is>
-          <t>19.355</t>
-        </is>
-      </c>
-      <c r="C72" s="19" t="inlineStr">
-        <is>
-          <t>8.484</t>
-        </is>
-      </c>
-      <c r="D72" s="19" t="inlineStr">
-        <is>
-          <t>180</t>
-        </is>
-      </c>
-      <c r="E72" s="19" t="inlineStr">
-        <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="F72" s="19" t="inlineStr">
-        <is>
-          <t>Fitted</t>
-        </is>
-      </c>
-      <c r="G72" s="19" t="inlineStr">
-        <is>
-          <t>AT24C256C-SSHL-T</t>
-        </is>
-      </c>
-      <c r="H72" s="19" t="inlineStr">
         <is>
           <t>SOIC127P600X265-8N (SOIC-8)</t>
         </is>

</xml_diff>